<commit_message>
add pull up and put down button
</commit_message>
<xml_diff>
--- a/kinimatics_ex.xlsx
+++ b/kinimatics_ex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projectPython\Scara_Robot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07143A93-B6A0-43A5-A584-308469BFEFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B53DD25B-9BC6-4C49-BAD9-024981C9317C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{F7D15F0B-DD29-4639-9934-56A6A717E228}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{F7D15F0B-DD29-4639-9934-56A6A717E228}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -245,15 +245,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>280148</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>9405</xdr:rowOff>
+      <xdr:colOff>197322</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>175057</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>369794</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>189619</xdr:rowOff>
+      <xdr:colOff>286968</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>164771</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -276,8 +276,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5221942" y="2676405"/>
-          <a:ext cx="6140823" cy="3609214"/>
+          <a:off x="5191735" y="3223057"/>
+          <a:ext cx="6218776" cy="3609214"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>